<commit_message>
Add offline/submission setup (no Google credentials needed)
- sample_emails.json: full synthetic email set (27 msgs) with personal
  addresses anonymized -> agent runs fully offline in manual mode.
- SUBMISSION.md: run guide for organizers (manual mode, temp LLM key, no
  credentials.json / gmail_token.pkl required).
- .env.example: default DATA_SOURCE_MODE=manual for submission/demo.
- Regenerated Report_Sample outputs from the offline run.

Verified: DATA_SOURCE_MODE=manual produces the full .docx report (all 7
initiatives updated from sample_emails.json) with no Gmail access.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Report_Sample/Initiatives tracker/Initiatives tracker thang 6-2026.xlsx
+++ b/Report_Sample/Initiatives tracker/Initiatives tracker thang 6-2026.xlsx
@@ -520,7 +520,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Thư. Trần Thị (2)</t>
+          <t>Persona 1</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -535,12 +535,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Jun-26</t>
+          <t>May-26</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Đã live trên production, mở luồng cho new user từ đầu tháng 6.</t>
+          <t>Đã live trên production từ 7/6 sau khi hoàn thành UAT và Risk sign off.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Thư. Trần Thị (2)</t>
+          <t>Persona 1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Đối tác yêu cầu support risk-based pricing API, delay thêm 6-8 tuần, dự kiến launch tháng 10.</t>
+          <t>Đối tác yêu cầu bắt buộc API risk-based pricing chưa nằm trong scope, dự kiến delay sang tháng 10.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Thư Trần</t>
+          <t>Persona 2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Model v1 Gini thấp hơn kỳ vọng (~0.2 vs 0.4), đang optimize, timeline Sep chưa đổi.</t>
+          <t>Model v1 đang chạy offline nhưng Gini thấp hơn kỳ vọng, team DS đang optimize nhưng chưa ảnh hưởng timeline.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Thư. Trần Thị (2)</t>
+          <t>Persona 3</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>UAT hoàn thành cuối tháng 5, deploy và go live ngày 7/6.</t>
+          <t>Đã live trên production từ 7/6 sau khi hoàn thành UAT và deploy.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Model đã deploy tháng 5, đang theo dõi hiệu quả thực tế và remediation tỷ lệ duyệt.</t>
+          <t>Model đã deploy tháng 5, đang trong quá trình remediation để khôi phục tỷ lệ duyệt.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Thư Trần</t>
+          <t>Persona 3</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Do resource Cashier full load, đồng ý deprioritize và back lại trong Q4.</t>
+          <t>Do team Cashier full load và performance test chưa ổn định, đã đồng ý deprioritize và reschedule sang Q4.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Thư Trần</t>
+          <t>Persona 2</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>DS ưu tiên init khác, chưa có resource để scoping, timeline chưa confirm.</t>
+          <t>Chưa thể bắt đầu scoping do team DS đang ưu tiên init optimize data model khác.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">

</xml_diff>

<commit_message>
Refresh Report_Sample with corrected June run (Excel closed)
Canonical tracker now reflects accurate extraction: #3 New modelling reads the
latest "Gini up to 0.3, near threshold"; #10 personalization new timing = Aug-26.
Forecast / Performance analysis / report .docx regenerated consistently.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Report_Sample/Initiatives tracker/Initiatives tracker thang 6-2026.xlsx
+++ b/Report_Sample/Initiatives tracker/Initiatives tracker thang 6-2026.xlsx
@@ -525,22 +525,20 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Live</t>
+          <t>On Track</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>May-26</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Đã live trên production từ đầu tháng 6, luồng thông và Risk đã sign off.</t>
+          <t>- Integration and UAT finished in 04/2026
+- Contract finalized in 04/2026
+- Ready to pilot in mid 05/2026 
+=&gt; %Eligible/Total +10pp vs Apr</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -590,7 +588,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Đối tác yêu cầu bắt buộc API risk-based pricing chưa nằm trong scope, dự kiến delay sang tháng 10.</t>
+          <t>Đối tác yêu cầu bắt buộc risk-based pricing API, cần thêm 6-8 tuần dev và UAT, timeline khả thi nhất là tháng 10.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -640,12 +638,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Model v1 đang optimize do Gini thấp hơn kỳ vọng, timeline tháng 9 chưa bị ảnh hưởng.</t>
+          <t>Model v1 đã được optimize, Gini tăng lên 0.3, team đang ở bước cuối để launch theo timeline tháng 9.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -690,7 +688,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Đã live trên production từ 7/6 sau khi fix edge case và hoàn thành UAT cuối tháng 5.</t>
+          <t>Đã live trên production từ 7/6 sau khi fix edge case eligibility và Risk sign off.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -748,7 +746,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Model đã deploy tháng 5, đang remediation do tỷ lệ duyệt tuyệt đối chưa đạt mục tiêu.</t>
+          <t>Model v-next đã deploy tháng 5, đạt mục tiêu +5pp Eligible và +10pp Approval, tuy nhiên AR tuyệt đối ~65% chưa đạt target 70% đang trong quá trình khắc phục.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -833,7 +831,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Do team Cashier full load và performance test chưa ổn định, đã đồng ý deprioritize và reschedule sang Q4.</t>
+          <t>Đã đồng ý deprioritize do team Cashier full load và performance test chưa ổn định, sẽ quay lại Q4 khi có resource.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -947,9 +945,14 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Không thể bắt đầu scoping do team DS đang ưu tiên init optimize model, timeline tháng 7 không khả thi.</t>
+          <t>Không thể kick off ngay tháng 6 do team DS đang ưu tiên init optimize model, cần 2 tháng để hoàn thiện sau khi model chạy positive.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">

</xml_diff>

<commit_message>
Email reading: a resolved blocker isn't a current blocker
Prompt now tells the model that when an older message said an initiative was
blocked/"cannot start" and a newer message says it is unblocked/"can kick off",
the details must describe the NEW state. Fixes #10 personalization details:
was "cannot kick off in June" (stale 15-Jun blocker) -> now "can kick off end
June (model ready), needs 2 months -> delayed to Aug-26".

Refresh Report_Sample + sample_emails.json accordingly.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Report_Sample/Initiatives tracker/Initiatives tracker thang 6-2026.xlsx
+++ b/Report_Sample/Initiatives tracker/Initiatives tracker thang 6-2026.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Đối tác yêu cầu bắt buộc risk-based pricing API, cần thêm 6-8 tuần dev và UAT, timeline khả thi nhất là tháng 10.</t>
+          <t>Partner yêu cầu bắt buộc risk-based pricing API, cần thêm 6-8 tuần dev và UAT, timeline khả thi nhất là tháng 10.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Model v-next đã deploy tháng 5, đạt mục tiêu +5pp Eligible và +10pp Approval, tuy nhiên AR tuyệt đối ~65% chưa đạt target 70% đang trong quá trình khắc phục.</t>
+          <t>Model v-next đã deploy tháng 5, đạt +5pp Eligible và +10pp approval, tuy nhiên absolute approval ~65% chưa đạt target 70% đang trong quá trình remediation.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Đã đồng ý deprioritize do team Cashier full load và performance test chưa ổn định, sẽ quay lại Q4 khi có resource.</t>
+          <t>Do team Cashier full load và performance test chưa ổn định, hai bên đồng ý deprioritize và sẽ quay lại trong Q4 khi có resource.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -952,12 +952,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Không thể kick off ngay tháng 6 do team DS đang ưu tiên init optimize model, cần 2 tháng để hoàn thiện sau khi model chạy positive.</t>
+          <t>Do team DS ưu tiên init optimize model, init này chưa thể scoping ngay, dự kiến kick off cuối tháng 6 và cần 2 tháng để hoàn thiện.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -1040,9 +1040,19 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Q4-2026</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Planning to begin Q3; creative &amp; budget not yet locked.</t>
+          <t>Vẫn chưa có cập nhật mới, kế hoạch bắt đầu Q3 với creative và budget chưa chốt.</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
2-pass thread→initiative mapping: merge same-initiative threads, fix #1/#2
Adds a cheap Pass-1 LLM call mapping each email thread to initiative No(s), then:
- MERGES threads that concern the same single initiative (e.g. "Partner 2 —
  onboarding" + "Onboard Partner A" -> #2) so the latest decision wins → #2 now
  reads the phased plan (Phase 1 ~Sep, 1M users; Phase 2 later).
- Leaves multi-initiative threads as-is (no cross-contamination) → #3/#10 stay correct.
- Completeness sweep: no-email, past-due, ready/deployed items roll to Live (Rule B)
  → #1 (ready-to-pilot May) becomes Live in June.
- max_tokens 8000 + _chat_json/_json_obj helpers (supports reasoning models too).

Verified stable: #1 Live, #2 Sep-26 phased, #3 On Track Sep-26, #10 Delay Aug-26.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Report_Sample/Initiatives tracker/Initiatives tracker thang 6-2026.xlsx
+++ b/Report_Sample/Initiatives tracker/Initiatives tracker thang 6-2026.xlsx
@@ -525,20 +525,22 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>On Track</t>
+          <t>Live</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>May-26</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>- Integration and UAT finished in 04/2026
-- Contract finalized in 04/2026
-- Ready to pilot in mid 05/2026 
-=&gt; %Eligible/Total +10pp vs Apr</t>
+          <t>Đã hoàn thành tích hợp và UAT vào tháng 4, sẵn sàng pilot giữa tháng 5, hiện đã đi vào hoạt động.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -583,12 +585,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Oct-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Partner yêu cầu bắt buộc risk-based pricing API, cần thêm 6-8 tuần dev và UAT, timeline khả thi nhất là tháng 10.</t>
+          <t>Đối tác đồng ý triển khai theo giai đoạn, nhưng cần thêm 2 tuần so với kế hoạch ban đầu (31/8), dự kiến Phase 1 vào tháng 9 với 1 triệu user.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -638,7 +640,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Model v1 đã được optimize, Gini tăng lên 0.3, team đang ở bước cuối để launch theo timeline tháng 9.</t>
+          <t>Mô hình v1 đã được tối ưu (Gini 0.3), đang ở bước cuối để tối ưu và dự kiến launch đúng kế hoạch tháng 9.</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -688,7 +690,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Đã live trên production từ 7/6 sau khi fix edge case eligibility và Risk sign off.</t>
+          <t>Đã hoàn thành UAT và deploy vào ngày 7/6, sản phẩm đã live trên production.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -746,7 +748,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Model v-next đã deploy tháng 5, đạt +5pp Eligible và +10pp approval, tuy nhiên absolute approval ~65% chưa đạt target 70% đang trong quá trình remediation.</t>
+          <t>Mô hình v-next đã được triển khai vào tháng 5, đạt mục tiêu tăng 5pp Eligible và 10pp Approval Rate, tuy nhiên tỷ lệ chấp nhận tuyệt đối đang ở mức 65%.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -789,6 +791,21 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Kênh traffic mới #1 đã được triển khai và đang hoạt động.</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -831,7 +848,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Do team Cashier full load và performance test chưa ổn định, hai bên đồng ý deprioritize và sẽ quay lại trong Q4 khi có resource.</t>
+          <t>Do team Cashier không có nguồn lực và vấn đề hiệu năng, initiative này đã được đồng ý deprioritize và sẽ xem xét lại vào Q4.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -874,6 +891,21 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Việc cải tiến layout Landing Page đã hoàn thành và đang hoạt động.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -910,6 +942,21 @@
           <t>No</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Việc đa dạng hóa sản phẩm đã hoàn thành và đang hoạt động.</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -952,12 +999,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Do team DS ưu tiên init optimize model, init này chưa thể scoping ngay, dự kiến kick off cuối tháng 6 và cần 2 tháng để hoàn thiện.</t>
+          <t>Do team DS ưu tiên tối ưu mô hình dữ liệu, việc scoping bị trì hoãn; dự kiến cần 2 tháng để hoàn thiện sau khi bắt đầu.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -997,12 +1044,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Q4/2026</t>
+          <t>Q4-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Low expected impact (+0.5pp); deprioritized vs higher-impact channel work; may revisit Q4.</t>
+          <t>Đã được deprioritize do tác động thấp, có thể xem xét lại vào Q4.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1099,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Vẫn chưa có cập nhật mới, kế hoạch bắt đầu Q3 với creative và budget chưa chốt.</t>
+          <t>Chưa bắt đầu, đang trong giai đoạn lập kế hoạch cho Q3 với ngân sách và sáng tạo chưa chốt.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">

</xml_diff>